<commit_message>
📊 Stock screener 2026-03-15
</commit_message>
<xml_diff>
--- a/output/stock_deviation_2026-03-15.xlsx
+++ b/output/stock_deviation_2026-03-15.xlsx
@@ -740,7 +740,7 @@
         <v>9.6</v>
       </c>
       <c r="Q2" s="8" t="n">
-        <v>816.578</v>
+        <v>816.574</v>
       </c>
       <c r="R2" s="9" t="n">
         <v>6514</v>
@@ -29197,7 +29197,7 @@
         <v>9.6</v>
       </c>
       <c r="Q2" s="8" t="n">
-        <v>816.578</v>
+        <v>816.574</v>
       </c>
       <c r="R2" s="9" t="n">
         <v>6514</v>
@@ -58035,7 +58035,7 @@
         <v>9.6</v>
       </c>
       <c r="Q2" s="8" t="n">
-        <v>816.578</v>
+        <v>816.574</v>
       </c>
       <c r="R2" s="9" t="n">
         <v>6514</v>

</xml_diff>